<commit_message>
Update overview page for standardized Excel columns
</commit_message>
<xml_diff>
--- a/data/Brand_Master.xlsx
+++ b/data/Brand_Master.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apparelme-my.sharepoint.com/personal/138925_appareluae_com/Documents/LS Retail - Masters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apparelme-my.sharepoint.com/personal/138925_appareluae_com/Documents/F&amp;B Sales Dashboard - Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9D9573E-55C1-48D2-AB5A-031BC2061E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{A9D9573E-55C1-48D2-AB5A-031BC2061E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37B55CDC-C350-498A-8A6D-90A5109D9A52}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3C0D9F61-7A1E-426B-B23D-A3F7CEAF51F9}"/>
+    <workbookView xWindow="8140" yWindow="1110" windowWidth="11760" windowHeight="6160" xr2:uid="{3C0D9F61-7A1E-426B-B23D-A3F7CEAF51F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Brand_Master_tbl" sheetId="1" r:id="rId1"/>
@@ -39,18 +39,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
-    <t>Brand_Sr_No</t>
-  </si>
-  <si>
-    <t>Brand_Name</t>
-  </si>
-  <si>
-    <t>Brand_Ora_Code</t>
-  </si>
-  <si>
-    <t>Brand_Code</t>
-  </si>
-  <si>
     <t>ALB</t>
   </si>
   <si>
@@ -87,9 +75,6 @@
     <t>NANDO'S</t>
   </si>
   <si>
-    <t>Brand_Desc</t>
-  </si>
-  <si>
     <t>Allo Beirut</t>
   </si>
   <si>
@@ -124,6 +109,21 @@
   </si>
   <si>
     <t>Sushi Library</t>
+  </si>
+  <si>
+    <t>brand_sr_no</t>
+  </si>
+  <si>
+    <t>brand_code</t>
+  </si>
+  <si>
+    <t>brand_name</t>
+  </si>
+  <si>
+    <t>brand_desc</t>
+  </si>
+  <si>
+    <t>brand_ora_code</t>
   </si>
 </sst>
 </file>
@@ -491,19 +491,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -511,13 +511,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1">
         <v>510013</v>
@@ -528,13 +528,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E3" s="1">
         <v>530001</v>
@@ -545,13 +545,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E4" s="1">
         <v>510005</v>
@@ -562,13 +562,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E5" s="1">
         <v>510003</v>
@@ -579,13 +579,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E6" s="1">
         <v>510006</v>
@@ -596,13 +596,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E7" s="1">
         <v>510012</v>
@@ -613,13 +613,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="E8" s="1">
         <v>530005</v>
@@ -630,13 +630,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E9" s="1">
         <v>510016</v>

</xml_diff>